<commit_message>
initial updates for 2026
</commit_message>
<xml_diff>
--- a/assets/schedule.xlsx
+++ b/assets/schedule.xlsx
@@ -5,10 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Schedule" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Full" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Short" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="18">
   <si>
     <t xml:space="preserve">Course
 Week</t>
@@ -211,37 +212,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -359,7 +360,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -370,7 +371,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>7</v>
@@ -381,7 +382,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>8</v>
@@ -392,7 +393,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>9</v>
@@ -409,7 +410,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>12</v>
@@ -420,7 +421,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>13</v>
@@ -431,7 +432,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>14</v>
@@ -442,7 +443,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>15</v>
@@ -456,13 +457,158 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>13</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="29.39"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="14.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>38</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <v>40</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>41</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>42</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>